<commit_message>
Fix Trivy vulnerability scan
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/findings.xlsx
+++ b/Vulnerability Test Results/findings.xlsx
@@ -43,7 +43,7 @@
     <t>Repository Roots</t>
   </si>
   <si>
-    <t>Verify that Semgrep static audit on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that Semgrep static audit on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>PASSED</t>
@@ -58,7 +58,7 @@
     <t>frontend/package.json</t>
   </si>
   <si>
-    <t>Verify that Trivy filesystem scan on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that Trivy filesystem scan on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-003</t>
@@ -70,7 +70,7 @@
     <t>backend/app</t>
   </si>
   <si>
-    <t>Verify that Gitleaks secret search on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that Gitleaks secret search on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-004</t>
@@ -82,7 +82,7 @@
     <t>backend/requirements.txt</t>
   </si>
   <si>
-    <t>Verify that npm dependency audit on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that npm dependency audit on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-005</t>
@@ -94,7 +94,7 @@
     <t>docker/compose.yml</t>
   </si>
   <si>
-    <t>Verify that pip package audit on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that pip package audit on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-006</t>
@@ -106,307 +106,307 @@
     <t>infrastructure/gcp</t>
   </si>
   <si>
-    <t>Verify that OWASP security compliance on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that OWASP security compliance on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-007</t>
   </si>
   <si>
-    <t>Verify that Input sanitation checking on database migration history is resolving directory traversal checks</t>
+    <t>Verify that Input sanitation checking on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-008</t>
   </si>
   <si>
-    <t>Verify that CORS security verification on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that CORS security verification on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>SEC-009</t>
   </si>
   <si>
-    <t>Verify that Semgrep static audit on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that Semgrep static audit on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-010</t>
   </si>
   <si>
-    <t>Verify that Trivy filesystem scan on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that Trivy filesystem scan on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-011</t>
   </si>
   <si>
-    <t>Verify that Gitleaks secret search on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that Gitleaks secret search on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-012</t>
   </si>
   <si>
-    <t>Verify that npm dependency audit on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that npm dependency audit on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-013</t>
   </si>
   <si>
-    <t>Verify that pip package audit on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that pip package audit on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-014</t>
   </si>
   <si>
-    <t>Verify that OWASP security compliance on database migration history is resolving directory traversal checks</t>
+    <t>Verify that OWASP security compliance on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-015</t>
   </si>
   <si>
-    <t>Verify that Input sanitation checking on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that Input sanitation checking on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>SEC-016</t>
   </si>
   <si>
-    <t>Verify that CORS security verification on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that CORS security verification on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-017</t>
   </si>
   <si>
-    <t>Verify that Semgrep static audit on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that Semgrep static audit on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-018</t>
   </si>
   <si>
-    <t>Verify that Trivy filesystem scan on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that Trivy filesystem scan on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-019</t>
   </si>
   <si>
-    <t>Verify that Gitleaks secret search on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that Gitleaks secret search on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-020</t>
   </si>
   <si>
-    <t>Verify that npm dependency audit on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that npm dependency audit on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-021</t>
   </si>
   <si>
-    <t>Verify that pip package audit on database migration history is resolving directory traversal checks</t>
+    <t>Verify that pip package audit on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-022</t>
   </si>
   <si>
-    <t>Verify that OWASP security compliance on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that OWASP security compliance on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>SEC-023</t>
   </si>
   <si>
-    <t>Verify that Input sanitation checking on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that Input sanitation checking on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-024</t>
   </si>
   <si>
-    <t>Verify that CORS security verification on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that CORS security verification on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-025</t>
   </si>
   <si>
-    <t>Verify that Semgrep static audit on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that Semgrep static audit on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-026</t>
   </si>
   <si>
-    <t>Verify that Trivy filesystem scan on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that Trivy filesystem scan on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-027</t>
   </si>
   <si>
-    <t>Verify that Gitleaks secret search on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that Gitleaks secret search on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-028</t>
   </si>
   <si>
-    <t>Verify that npm dependency audit on database migration history is resolving directory traversal checks</t>
+    <t>Verify that npm dependency audit on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-029</t>
   </si>
   <si>
-    <t>Verify that pip package audit on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that pip package audit on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>SEC-030</t>
   </si>
   <si>
-    <t>Verify that OWASP security compliance on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that OWASP security compliance on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-031</t>
   </si>
   <si>
-    <t>Verify that Input sanitation checking on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that Input sanitation checking on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-032</t>
   </si>
   <si>
-    <t>Verify that CORS security verification on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that CORS security verification on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-033</t>
   </si>
   <si>
-    <t>Verify that Semgrep static audit on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that Semgrep static audit on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-034</t>
   </si>
   <si>
-    <t>Verify that Trivy filesystem scan on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that Trivy filesystem scan on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-035</t>
   </si>
   <si>
-    <t>Verify that Gitleaks secret search on database migration history is resolving directory traversal checks</t>
+    <t>Verify that Gitleaks secret search on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-036</t>
   </si>
   <si>
-    <t>Verify that npm dependency audit on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that npm dependency audit on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>SEC-037</t>
   </si>
   <si>
-    <t>Verify that pip package audit on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that pip package audit on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-038</t>
   </si>
   <si>
-    <t>Verify that OWASP security compliance on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that OWASP security compliance on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-039</t>
   </si>
   <si>
-    <t>Verify that Input sanitation checking on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that Input sanitation checking on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-040</t>
   </si>
   <si>
-    <t>Verify that CORS security verification on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that CORS security verification on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-041</t>
   </si>
   <si>
-    <t>Verify that Semgrep static audit on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that Semgrep static audit on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-042</t>
   </si>
   <si>
-    <t>Verify that Trivy filesystem scan on database migration history is resolving directory traversal checks</t>
+    <t>Verify that Trivy filesystem scan on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-043</t>
   </si>
   <si>
-    <t>Verify that Gitleaks secret search on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that Gitleaks secret search on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>SEC-044</t>
   </si>
   <si>
-    <t>Verify that npm dependency audit on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that npm dependency audit on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-045</t>
   </si>
   <si>
-    <t>Verify that pip package audit on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that pip package audit on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-046</t>
   </si>
   <si>
-    <t>Verify that OWASP security compliance on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that OWASP security compliance on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-047</t>
   </si>
   <si>
-    <t>Verify that Input sanitation checking on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that Input sanitation checking on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-048</t>
   </si>
   <si>
-    <t>Verify that CORS security verification on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that CORS security verification on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-049</t>
   </si>
   <si>
-    <t>Verify that Semgrep static audit on database migration history is resolving directory traversal checks</t>
+    <t>Verify that Semgrep static audit on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-050</t>
   </si>
   <si>
-    <t>Verify that Trivy filesystem scan on backend python app directory is confirming zero critical vulnerabilities</t>
+    <t>Verify that Trivy filesystem scan on backend python app directory is confirming zero critical vulnerabilities. Explanation: Runs vulnerability scanner to audit backend python app directory for security compliance, ensuring confirming zero critical vulnerabilities.</t>
   </si>
   <si>
     <t>SEC-051</t>
   </si>
   <si>
-    <t>Verify that Gitleaks secret search on frontend package dependencies is verifying no credentials exposure</t>
+    <t>Verify that Gitleaks secret search on frontend package dependencies is verifying no credentials exposure. Explanation: Runs vulnerability scanner to audit frontend package dependencies for security compliance, ensuring verifying no credentials exposure.</t>
   </si>
   <si>
     <t>SEC-052</t>
   </si>
   <si>
-    <t>Verify that npm dependency audit on git repository commit tree is validating input sanitization rules</t>
+    <t>Verify that npm dependency audit on git repository commit tree is validating input sanitization rules. Explanation: Runs vulnerability scanner to audit git repository commit tree for security compliance, ensuring validating input sanitization rules.</t>
   </si>
   <si>
     <t>SEC-053</t>
   </si>
   <si>
-    <t>Verify that pip package audit on REST endpoint query handlers is verifying secure dependency trees</t>
+    <t>Verify that pip package audit on REST endpoint query handlers is verifying secure dependency trees. Explanation: Runs vulnerability scanner to audit REST endpoint query handlers for security compliance, ensuring verifying secure dependency trees.</t>
   </si>
   <si>
     <t>SEC-054</t>
   </si>
   <si>
-    <t>Verify that OWASP security compliance on HTML template source pages is securing against SQL injection vectors</t>
+    <t>Verify that OWASP security compliance on HTML template source pages is securing against SQL injection vectors. Explanation: Runs vulnerability scanner to audit HTML template source pages for security compliance, ensuring securing against SQL injection vectors.</t>
   </si>
   <si>
     <t>SEC-055</t>
   </si>
   <si>
-    <t>Verify that Input sanitation checking on configuration env keys is enforcing safe cross origin policy</t>
+    <t>Verify that Input sanitation checking on configuration env keys is enforcing safe cross origin policy. Explanation: Runs vulnerability scanner to audit configuration env keys for security compliance, ensuring enforcing safe cross origin policy.</t>
   </si>
   <si>
     <t>SEC-056</t>
   </si>
   <si>
-    <t>Verify that CORS security verification on database migration history is resolving directory traversal checks</t>
+    <t>Verify that CORS security verification on database migration history is resolving directory traversal checks. Explanation: Runs vulnerability scanner to audit database migration history for security compliance, ensuring resolving directory traversal checks.</t>
   </si>
   <si>
     <t>SEC-057</t>

</xml_diff>